<commit_message>
done with RE SV
</commit_message>
<xml_diff>
--- a/БД/funcs/VV_LVALH.xlsx
+++ b/БД/funcs/VV_LVALH.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="812" uniqueCount="233">
   <si>
     <t>Modbus RTU</t>
   </si>
@@ -462,15 +462,6 @@
     <t>OvrlExtSignFrmSignAssem</t>
   </si>
   <si>
-    <t>Положение переключателя аварийной деблокировки</t>
-  </si>
-  <si>
-    <t>Полож.пер.ав.дебл.</t>
-  </si>
-  <si>
-    <t>SwPosOfEmergUnblk</t>
-  </si>
-  <si>
     <t>Внутренняя неисправность</t>
   </si>
   <si>
@@ -713,12 +704,33 @@
   <si>
     <t>Сраб УРОВ на себя</t>
   </si>
+  <si>
+    <t>input</t>
+  </si>
+  <si>
+    <t>Положение переключателя аварийной деблокировки 1</t>
+  </si>
+  <si>
+    <t>Полож.пер.ав.дебл.1</t>
+  </si>
+  <si>
+    <t>SwPosOfEmergUnblk1</t>
+  </si>
+  <si>
+    <t>Положение переключателя аварийной деблокировки 2</t>
+  </si>
+  <si>
+    <t>Полож.пер.ав.дебл.2</t>
+  </si>
+  <si>
+    <t>SwPosOfEmergUnblk2</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -791,8 +803,15 @@
       <family val="2"/>
       <charset val="204"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -825,7 +844,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -891,7 +916,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1053,12 +1078,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1073,15 +1092,91 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1363,7 +1458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:XEY131"/>
+  <dimension ref="A1:XEY132"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="5.65" customHeight="1" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.140625" style="1" bestFit="1" customWidth="1"/>
@@ -1455,15 +1550,15 @@
       <c r="AW1" s="6"/>
       <c r="AX1" s="6"/>
       <c r="AY1" s="8"/>
-      <c r="AZ1" s="59" t="s">
+      <c r="AZ1" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="BA1" s="60"/>
-      <c r="BB1" s="60"/>
-      <c r="BC1" s="60"/>
-      <c r="BD1" s="60"/>
-      <c r="BE1" s="60"/>
-      <c r="BF1" s="60"/>
+      <c r="BA1" s="67"/>
+      <c r="BB1" s="67"/>
+      <c r="BC1" s="67"/>
+      <c r="BD1" s="67"/>
+      <c r="BE1" s="67"/>
+      <c r="BF1" s="67"/>
     </row>
     <row r="2" spans="1:16379" s="17" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
@@ -1607,14 +1702,14 @@
       <c r="AU2" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="AV2" s="65" t="s">
-        <v>223</v>
-      </c>
-      <c r="AW2" s="65" t="s">
-        <v>224</v>
-      </c>
-      <c r="AX2" s="65" t="s">
-        <v>225</v>
+      <c r="AV2" s="63" t="s">
+        <v>220</v>
+      </c>
+      <c r="AW2" s="63" t="s">
+        <v>221</v>
+      </c>
+      <c r="AX2" s="63" t="s">
+        <v>222</v>
       </c>
       <c r="AY2" s="14"/>
       <c r="AZ2" s="13" t="s">
@@ -17962,126 +18057,126 @@
       <c r="XEX2" s="1"/>
       <c r="XEY2" s="1"/>
     </row>
-    <row r="3" spans="1:16379" s="44" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="46"/>
-      <c r="B3" s="67" t="s">
-        <v>226</v>
-      </c>
-      <c r="C3" s="47"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="48" t="s">
+    <row r="3" spans="1:16379" s="82" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="68"/>
+      <c r="B3" s="68" t="s">
+        <v>223</v>
+      </c>
+      <c r="C3" s="69"/>
+      <c r="D3" s="70"/>
+      <c r="E3" s="71" t="s">
         <v>60</v>
       </c>
-      <c r="F3" s="48" t="s">
+      <c r="F3" s="71" t="s">
         <v>60</v>
       </c>
-      <c r="G3" s="48" t="s">
+      <c r="G3" s="71" t="s">
         <v>60</v>
       </c>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48">
-        <f t="shared" ref="I3:I40" si="0">LEN(F3)</f>
+      <c r="H3" s="71"/>
+      <c r="I3" s="71">
+        <f t="shared" ref="I3:I41" si="0">LEN(F3)</f>
         <v>15</v>
       </c>
-      <c r="J3" s="48" t="str">
-        <f t="shared" ref="J3:J40" si="1">IF(LEN(F3)&lt;=$J$1,F3,"")</f>
+      <c r="J3" s="71" t="str">
+        <f t="shared" ref="J3:J41" si="1">IF(LEN(F3)&lt;=$J$1,F3,"")</f>
         <v>Вывод терминала</v>
       </c>
-      <c r="K3" s="46" t="s">
+      <c r="K3" s="68" t="s">
         <v>61</v>
       </c>
-      <c r="L3" s="49" t="s">
+      <c r="L3" s="72" t="s">
         <v>62</v>
       </c>
-      <c r="M3" s="47" t="s">
+      <c r="M3" s="69" t="s">
         <v>63</v>
       </c>
-      <c r="N3" s="47" t="s">
+      <c r="N3" s="69" t="s">
         <v>64</v>
       </c>
-      <c r="O3" s="47"/>
-      <c r="P3" s="50"/>
-      <c r="Q3" s="50"/>
-      <c r="R3" s="47" t="s">
+      <c r="O3" s="69"/>
+      <c r="P3" s="73"/>
+      <c r="Q3" s="73"/>
+      <c r="R3" s="69" t="s">
         <v>65</v>
       </c>
-      <c r="S3" s="47" t="s">
+      <c r="S3" s="69" t="s">
         <v>65</v>
       </c>
-      <c r="T3" s="47" t="s">
+      <c r="T3" s="69" t="s">
         <v>65</v>
       </c>
-      <c r="U3" s="47" t="s">
+      <c r="U3" s="69" t="s">
         <v>65</v>
       </c>
-      <c r="V3" s="47"/>
-      <c r="W3" s="47"/>
-      <c r="X3" s="47" t="s">
+      <c r="V3" s="69"/>
+      <c r="W3" s="69"/>
+      <c r="X3" s="69" t="s">
         <v>65</v>
       </c>
-      <c r="Y3" s="47">
+      <c r="Y3" s="69">
         <v>0</v>
       </c>
-      <c r="Z3" s="51"/>
-      <c r="AA3" s="52">
+      <c r="Z3" s="74"/>
+      <c r="AA3" s="75">
         <v>0</v>
       </c>
-      <c r="AB3" s="52"/>
-      <c r="AC3" s="52"/>
-      <c r="AD3" s="52"/>
-      <c r="AE3" s="52"/>
-      <c r="AF3" s="52">
+      <c r="AB3" s="75"/>
+      <c r="AC3" s="75"/>
+      <c r="AD3" s="75"/>
+      <c r="AE3" s="75"/>
+      <c r="AF3" s="75">
         <v>0</v>
       </c>
-      <c r="AG3" s="52">
+      <c r="AG3" s="75">
         <v>0</v>
       </c>
-      <c r="AH3" s="52">
+      <c r="AH3" s="75">
         <v>0</v>
       </c>
-      <c r="AI3" s="53"/>
-      <c r="AJ3" s="54"/>
-      <c r="AK3" s="54"/>
-      <c r="AL3" s="54"/>
-      <c r="AM3" s="54"/>
-      <c r="AN3" s="54"/>
-      <c r="AO3" s="54"/>
-      <c r="AP3" s="54"/>
-      <c r="AQ3" s="54"/>
-      <c r="AR3" s="52">
+      <c r="AI3" s="76"/>
+      <c r="AJ3" s="77"/>
+      <c r="AK3" s="77"/>
+      <c r="AL3" s="77"/>
+      <c r="AM3" s="77"/>
+      <c r="AN3" s="77"/>
+      <c r="AO3" s="77"/>
+      <c r="AP3" s="77"/>
+      <c r="AQ3" s="77"/>
+      <c r="AR3" s="75">
         <v>0</v>
       </c>
-      <c r="AS3" s="52">
+      <c r="AS3" s="75">
         <v>0</v>
       </c>
-      <c r="AT3" s="69">
+      <c r="AT3" s="75">
         <v>1</v>
       </c>
-      <c r="AU3" s="52">
+      <c r="AU3" s="75">
         <v>0</v>
       </c>
-      <c r="AV3" s="69">
+      <c r="AV3" s="75">
         <v>1</v>
       </c>
-      <c r="AW3" s="69">
+      <c r="AW3" s="75">
         <v>1</v>
       </c>
-      <c r="AX3" s="69">
+      <c r="AX3" s="75">
         <v>1</v>
       </c>
-      <c r="AY3" s="52"/>
-      <c r="AZ3" s="50"/>
-      <c r="BA3" s="52"/>
-      <c r="BB3" s="52"/>
-      <c r="BC3" s="55"/>
-      <c r="BD3" s="52"/>
-      <c r="BE3" s="56"/>
-      <c r="BF3" s="52"/>
-      <c r="BG3" s="57" t="str">
-        <f t="shared" ref="BG3:BG40" si="2">CONCATENATE("description: """,F3,"""", ", ", "note: """,E3,"""",", ","group: """, B3, """",", ","minValue: ", S3,", ","maxValue: ", T3,", ","step: ", U3,", ","units: """, R3, """",", ","defaultValue: ", X3,", ","eventRegistration: ", Y3,)</f>
+      <c r="AY3" s="75"/>
+      <c r="AZ3" s="73"/>
+      <c r="BA3" s="75"/>
+      <c r="BB3" s="75"/>
+      <c r="BC3" s="78"/>
+      <c r="BD3" s="75"/>
+      <c r="BE3" s="79"/>
+      <c r="BF3" s="75"/>
+      <c r="BG3" s="80" t="str">
+        <f t="shared" ref="BG3:BG41" si="2">CONCATENATE("description: """,F3,"""", ", ", "note: """,E3,"""",", ","group: """, B3, """",", ","minValue: ", S3,", ","maxValue: ", T3,", ","step: ", U3,", ","units: """, R3, """",", ","defaultValue: ", X3,", ","eventRegistration: ", Y3,)</f>
         <v>description: "Вывод терминала", note: "Вывод терминала", group: "control", minValue: null, maxValue: null, step: null, units: "null", defaultValue: null, eventRegistration: 0</v>
       </c>
-      <c r="BH3" s="58"/>
+      <c r="BH3" s="81"/>
     </row>
     <row r="4" spans="1:16379" s="44" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="46"/>
@@ -18182,7 +18277,7 @@
         <v>0</v>
       </c>
       <c r="AV4" s="52">
-        <f t="shared" ref="AV3:AV40" si="3">BIN2DEC(CONCATENATE(0,0,0,0,AR4,AS4,AT4,AU4))</f>
+        <f t="shared" ref="AV4:AV41" si="3">BIN2DEC(CONCATENATE(0,0,0,0,AR4,AS4,AT4,AU4))</f>
         <v>0</v>
       </c>
       <c r="AW4" s="52">
@@ -19311,13 +19406,13 @@
       <c r="C14" s="47"/>
       <c r="D14" s="45"/>
       <c r="E14" s="48" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="F14" s="48" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="G14" s="48" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="H14" s="48"/>
       <c r="I14" s="48">
@@ -19329,7 +19424,7 @@
         <v>Ср.сигн. ЗП</v>
       </c>
       <c r="K14" s="46" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="L14" s="49" t="s">
         <v>62</v>
@@ -19433,13 +19528,13 @@
       <c r="C15" s="47"/>
       <c r="D15" s="45"/>
       <c r="E15" s="48" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="F15" s="48" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="G15" s="48" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="H15" s="48"/>
       <c r="I15" s="48">
@@ -19451,7 +19546,7 @@
         <v>Ср.сигн. ЗМН 1ст.</v>
       </c>
       <c r="K15" s="46" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="L15" s="49" t="s">
         <v>62</v>
@@ -19555,13 +19650,13 @@
       <c r="C16" s="47"/>
       <c r="D16" s="45"/>
       <c r="E16" s="48" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="F16" s="48" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G16" s="48" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="H16" s="48"/>
       <c r="I16" s="48">
@@ -19573,7 +19668,7 @@
         <v>Ср.сигн. ЗМН 2ст.</v>
       </c>
       <c r="K16" s="46" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="L16" s="49" t="s">
         <v>62</v>
@@ -20043,13 +20138,13 @@
       <c r="C20" s="47"/>
       <c r="D20" s="45"/>
       <c r="E20" s="48" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="F20" s="48" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="G20" s="48" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="H20" s="48"/>
       <c r="I20" s="48">
@@ -20061,7 +20156,7 @@
         <v>Задержка включ. АПВ</v>
       </c>
       <c r="K20" s="46" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="L20" s="49" t="s">
         <v>62</v>
@@ -20165,13 +20260,13 @@
       <c r="C21" s="47"/>
       <c r="D21" s="45"/>
       <c r="E21" s="48" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="F21" s="48" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="G21" s="48" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="H21" s="48"/>
       <c r="I21" s="48">
@@ -20287,13 +20382,13 @@
       <c r="C22" s="47"/>
       <c r="D22" s="45"/>
       <c r="E22" s="48" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F22" s="48" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="G22" s="48" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H22" s="48"/>
       <c r="I22" s="48">
@@ -20896,14 +20991,14 @@
       </c>
       <c r="C27" s="47"/>
       <c r="D27" s="45"/>
-      <c r="E27" s="68" t="s">
-        <v>227</v>
-      </c>
-      <c r="F27" s="68" t="s">
-        <v>228</v>
-      </c>
-      <c r="G27" s="68" t="s">
-        <v>228</v>
+      <c r="E27" s="65" t="s">
+        <v>224</v>
+      </c>
+      <c r="F27" s="65" t="s">
+        <v>225</v>
+      </c>
+      <c r="G27" s="65" t="s">
+        <v>225</v>
       </c>
       <c r="H27" s="48"/>
       <c r="I27" s="48">
@@ -21385,13 +21480,13 @@
       <c r="C31" s="47"/>
       <c r="D31" s="45"/>
       <c r="E31" s="48" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="F31" s="48" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="G31" s="48" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="H31" s="48"/>
       <c r="I31" s="48">
@@ -21403,7 +21498,7 @@
         <v>Зад. вкл от ВНР</v>
       </c>
       <c r="K31" s="46" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="L31" s="49" t="s">
         <v>62</v>
@@ -21507,13 +21602,13 @@
       <c r="C32" s="47"/>
       <c r="D32" s="45"/>
       <c r="E32" s="48" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="F32" s="48" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="G32" s="48" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="H32" s="48"/>
       <c r="I32" s="48">
@@ -21525,7 +21620,7 @@
         <v>Зад. вкл от ЛВ ВНР</v>
       </c>
       <c r="K32" s="46" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="L32" s="49" t="s">
         <v>62</v>
@@ -22353,290 +22448,371 @@
       </c>
       <c r="BH38" s="30"/>
     </row>
-    <row r="39" spans="1:60" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="18"/>
-      <c r="B39" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="C39" s="19"/>
-      <c r="D39" s="20"/>
-      <c r="E39" s="21" t="s">
-        <v>145</v>
-      </c>
-      <c r="F39" s="21" t="s">
-        <v>146</v>
-      </c>
-      <c r="G39" s="21" t="s">
-        <v>146</v>
-      </c>
-      <c r="H39" s="21"/>
-      <c r="I39" s="48">
+    <row r="39" spans="1:60" s="95" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="83"/>
+      <c r="B39" s="83" t="s">
+        <v>226</v>
+      </c>
+      <c r="C39" s="84"/>
+      <c r="D39" s="85"/>
+      <c r="E39" s="86" t="s">
+        <v>227</v>
+      </c>
+      <c r="F39" s="86" t="s">
+        <v>228</v>
+      </c>
+      <c r="G39" s="86" t="s">
+        <v>228</v>
+      </c>
+      <c r="H39" s="86"/>
+      <c r="I39" s="86">
         <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-      <c r="J39" s="48" t="str">
+        <v>19</v>
+      </c>
+      <c r="J39" s="86" t="str">
         <f t="shared" si="1"/>
-        <v>Полож.пер.ав.дебл.</v>
-      </c>
-      <c r="K39" s="18" t="s">
-        <v>147</v>
-      </c>
-      <c r="L39" s="22" t="s">
+        <v>Полож.пер.ав.дебл.1</v>
+      </c>
+      <c r="K39" s="83" t="s">
+        <v>229</v>
+      </c>
+      <c r="L39" s="87" t="s">
         <v>62</v>
       </c>
-      <c r="M39" s="19" t="s">
+      <c r="M39" s="84" t="s">
         <v>63</v>
       </c>
-      <c r="N39" s="19" t="s">
+      <c r="N39" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="O39" s="19"/>
-      <c r="P39" s="23"/>
-      <c r="Q39" s="23"/>
-      <c r="R39" s="19" t="s">
+      <c r="O39" s="84"/>
+      <c r="P39" s="88"/>
+      <c r="Q39" s="88"/>
+      <c r="R39" s="84" t="s">
         <v>65</v>
       </c>
-      <c r="S39" s="19" t="s">
+      <c r="S39" s="84" t="s">
         <v>65</v>
       </c>
-      <c r="T39" s="19" t="s">
+      <c r="T39" s="84" t="s">
         <v>65</v>
       </c>
-      <c r="U39" s="19" t="s">
+      <c r="U39" s="84" t="s">
         <v>65</v>
       </c>
-      <c r="V39" s="19"/>
-      <c r="W39" s="19"/>
-      <c r="X39" s="19" t="s">
+      <c r="V39" s="84"/>
+      <c r="W39" s="84"/>
+      <c r="X39" s="84" t="s">
         <v>65</v>
       </c>
-      <c r="Y39" s="19">
+      <c r="Y39" s="84">
         <v>0</v>
       </c>
-      <c r="Z39" s="24"/>
-      <c r="AA39" s="25">
+      <c r="Z39" s="89"/>
+      <c r="AA39" s="90">
         <v>0</v>
       </c>
-      <c r="AB39" s="25"/>
-      <c r="AC39" s="25"/>
-      <c r="AD39" s="25"/>
-      <c r="AE39" s="25"/>
-      <c r="AF39" s="25">
+      <c r="AB39" s="90"/>
+      <c r="AC39" s="90"/>
+      <c r="AD39" s="90"/>
+      <c r="AE39" s="90"/>
+      <c r="AF39" s="90">
         <v>0</v>
       </c>
-      <c r="AG39" s="25">
+      <c r="AG39" s="90">
         <v>0</v>
       </c>
-      <c r="AH39" s="25">
+      <c r="AH39" s="90">
         <v>0</v>
       </c>
-      <c r="AI39" s="8"/>
-      <c r="AJ39" s="26"/>
-      <c r="AK39" s="26"/>
-      <c r="AL39" s="26"/>
-      <c r="AM39" s="26"/>
-      <c r="AN39" s="26"/>
-      <c r="AO39" s="26"/>
-      <c r="AP39" s="26"/>
-      <c r="AQ39" s="26"/>
-      <c r="AR39" s="25">
+      <c r="AI39" s="91"/>
+      <c r="AJ39" s="92"/>
+      <c r="AK39" s="92"/>
+      <c r="AL39" s="92"/>
+      <c r="AM39" s="92"/>
+      <c r="AN39" s="92"/>
+      <c r="AO39" s="92"/>
+      <c r="AP39" s="92"/>
+      <c r="AQ39" s="92"/>
+      <c r="AR39" s="90">
         <v>0</v>
       </c>
-      <c r="AS39" s="25">
+      <c r="AS39" s="90">
         <v>0</v>
       </c>
-      <c r="AT39" s="25">
+      <c r="AT39" s="90">
         <v>0</v>
       </c>
-      <c r="AU39" s="25">
+      <c r="AU39" s="90">
         <v>0</v>
       </c>
-      <c r="AV39" s="52">
+      <c r="AV39" s="90">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AW39" s="52">
+      <c r="AW39" s="90">
         <v>0</v>
       </c>
-      <c r="AX39" s="52">
+      <c r="AX39" s="90">
         <v>0</v>
       </c>
-      <c r="AY39" s="25"/>
-      <c r="AZ39" s="23"/>
-      <c r="BA39" s="25"/>
-      <c r="BB39" s="25"/>
-      <c r="BC39" s="27"/>
-      <c r="BD39" s="25"/>
-      <c r="BE39" s="28"/>
-      <c r="BF39" s="25"/>
-      <c r="BG39" s="57" t="str">
+      <c r="AY39" s="90"/>
+      <c r="AZ39" s="88"/>
+      <c r="BA39" s="90"/>
+      <c r="BB39" s="90"/>
+      <c r="BC39" s="90"/>
+      <c r="BD39" s="90"/>
+      <c r="BE39" s="90"/>
+      <c r="BF39" s="90"/>
+      <c r="BG39" s="93" t="str">
         <f t="shared" si="2"/>
-        <v>description: "Полож.пер.ав.дебл.", note: "Положение переключателя аварийной деблокировки", group: "measurement", minValue: null, maxValue: null, step: null, units: "null", defaultValue: null, eventRegistration: 0</v>
-      </c>
-      <c r="BH39" s="30"/>
+        <v>description: "Полож.пер.ав.дебл.1", note: "Положение переключателя аварийной деблокировки 1", group: "input", minValue: null, maxValue: null, step: null, units: "null", defaultValue: null, eventRegistration: 0</v>
+      </c>
+      <c r="BH39" s="94"/>
     </row>
-    <row r="40" spans="1:60" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="18"/>
-      <c r="B40" s="18" t="s">
+    <row r="40" spans="1:60" s="95" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="83"/>
+      <c r="B40" s="83" t="s">
+        <v>226</v>
+      </c>
+      <c r="C40" s="84"/>
+      <c r="D40" s="85"/>
+      <c r="E40" s="86" t="s">
+        <v>230</v>
+      </c>
+      <c r="F40" s="86" t="s">
+        <v>231</v>
+      </c>
+      <c r="G40" s="86" t="s">
+        <v>231</v>
+      </c>
+      <c r="H40" s="86"/>
+      <c r="I40" s="86">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="J40" s="86" t="str">
+        <f t="shared" si="1"/>
+        <v>Полож.пер.ав.дебл.2</v>
+      </c>
+      <c r="K40" s="83" t="s">
+        <v>232</v>
+      </c>
+      <c r="L40" s="87" t="s">
+        <v>62</v>
+      </c>
+      <c r="M40" s="84" t="s">
+        <v>63</v>
+      </c>
+      <c r="N40" s="84" t="s">
+        <v>64</v>
+      </c>
+      <c r="O40" s="84"/>
+      <c r="P40" s="88"/>
+      <c r="Q40" s="88"/>
+      <c r="R40" s="84" t="s">
+        <v>65</v>
+      </c>
+      <c r="S40" s="84" t="s">
+        <v>65</v>
+      </c>
+      <c r="T40" s="84" t="s">
+        <v>65</v>
+      </c>
+      <c r="U40" s="84" t="s">
+        <v>65</v>
+      </c>
+      <c r="V40" s="84"/>
+      <c r="W40" s="84"/>
+      <c r="X40" s="84" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y40" s="84">
+        <v>0</v>
+      </c>
+      <c r="Z40" s="89"/>
+      <c r="AA40" s="90">
+        <v>0</v>
+      </c>
+      <c r="AB40" s="90"/>
+      <c r="AC40" s="90"/>
+      <c r="AD40" s="90"/>
+      <c r="AE40" s="90"/>
+      <c r="AF40" s="90">
+        <v>0</v>
+      </c>
+      <c r="AG40" s="90">
+        <v>0</v>
+      </c>
+      <c r="AH40" s="90">
+        <v>0</v>
+      </c>
+      <c r="AI40" s="91"/>
+      <c r="AJ40" s="92"/>
+      <c r="AK40" s="92"/>
+      <c r="AL40" s="92"/>
+      <c r="AM40" s="92"/>
+      <c r="AN40" s="92"/>
+      <c r="AO40" s="92"/>
+      <c r="AP40" s="92"/>
+      <c r="AQ40" s="92"/>
+      <c r="AR40" s="90">
+        <v>0</v>
+      </c>
+      <c r="AS40" s="90">
+        <v>0</v>
+      </c>
+      <c r="AT40" s="90">
+        <v>0</v>
+      </c>
+      <c r="AU40" s="90">
+        <v>0</v>
+      </c>
+      <c r="AV40" s="90">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AW40" s="90">
+        <v>0</v>
+      </c>
+      <c r="AX40" s="90">
+        <v>0</v>
+      </c>
+      <c r="AY40" s="90"/>
+      <c r="AZ40" s="88"/>
+      <c r="BA40" s="90"/>
+      <c r="BB40" s="90"/>
+      <c r="BC40" s="90"/>
+      <c r="BD40" s="90"/>
+      <c r="BE40" s="90"/>
+      <c r="BF40" s="90"/>
+      <c r="BG40" s="93" t="str">
+        <f t="shared" si="2"/>
+        <v>description: "Полож.пер.ав.дебл.2", note: "Положение переключателя аварийной деблокировки 2", group: "input", minValue: null, maxValue: null, step: null, units: "null", defaultValue: null, eventRegistration: 0</v>
+      </c>
+      <c r="BH40" s="94"/>
+    </row>
+    <row r="41" spans="1:60" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="18"/>
+      <c r="B41" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="C40" s="19"/>
-      <c r="D40" s="20"/>
-      <c r="E40" s="21" t="s">
-        <v>148</v>
-      </c>
-      <c r="F40" s="21" t="s">
-        <v>149</v>
-      </c>
-      <c r="G40" s="21" t="s">
-        <v>149</v>
-      </c>
-      <c r="H40" s="21"/>
-      <c r="I40" s="48">
+      <c r="C41" s="19"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="21" t="s">
+        <v>145</v>
+      </c>
+      <c r="F41" s="21" t="s">
+        <v>146</v>
+      </c>
+      <c r="G41" s="21" t="s">
+        <v>146</v>
+      </c>
+      <c r="H41" s="21"/>
+      <c r="I41" s="48">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="J40" s="48" t="str">
+      <c r="J41" s="48" t="str">
         <f t="shared" si="1"/>
         <v>IRF</v>
       </c>
-      <c r="K40" s="18" t="s">
-        <v>150</v>
-      </c>
-      <c r="L40" s="22" t="s">
+      <c r="K41" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="L41" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="M40" s="19" t="s">
+      <c r="M41" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="N40" s="19" t="s">
+      <c r="N41" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="O40" s="19"/>
-      <c r="P40" s="23"/>
-      <c r="Q40" s="23"/>
-      <c r="R40" s="19" t="s">
+      <c r="O41" s="19"/>
+      <c r="P41" s="23"/>
+      <c r="Q41" s="23"/>
+      <c r="R41" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="S40" s="19" t="s">
+      <c r="S41" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="T40" s="19" t="s">
+      <c r="T41" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="U40" s="19" t="s">
+      <c r="U41" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="V40" s="19"/>
-      <c r="W40" s="19"/>
-      <c r="X40" s="19" t="s">
+      <c r="V41" s="19"/>
+      <c r="W41" s="19"/>
+      <c r="X41" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="Y40" s="19">
+      <c r="Y41" s="19">
         <v>0</v>
       </c>
-      <c r="Z40" s="24"/>
-      <c r="AA40" s="25">
+      <c r="Z41" s="24"/>
+      <c r="AA41" s="25">
         <v>0</v>
       </c>
-      <c r="AB40" s="25"/>
-      <c r="AC40" s="25"/>
-      <c r="AD40" s="25"/>
-      <c r="AE40" s="25"/>
-      <c r="AF40" s="25">
+      <c r="AB41" s="25"/>
+      <c r="AC41" s="25"/>
+      <c r="AD41" s="25"/>
+      <c r="AE41" s="25"/>
+      <c r="AF41" s="25">
         <v>0</v>
       </c>
-      <c r="AG40" s="25">
+      <c r="AG41" s="25">
         <v>0</v>
       </c>
-      <c r="AH40" s="25">
+      <c r="AH41" s="25">
         <v>0</v>
       </c>
-      <c r="AI40" s="8"/>
-      <c r="AJ40" s="26"/>
-      <c r="AK40" s="26"/>
-      <c r="AL40" s="26"/>
-      <c r="AM40" s="26"/>
-      <c r="AN40" s="26"/>
-      <c r="AO40" s="26"/>
-      <c r="AP40" s="26"/>
-      <c r="AQ40" s="26"/>
-      <c r="AR40" s="25">
+      <c r="AI41" s="8"/>
+      <c r="AJ41" s="26"/>
+      <c r="AK41" s="26"/>
+      <c r="AL41" s="26"/>
+      <c r="AM41" s="26"/>
+      <c r="AN41" s="26"/>
+      <c r="AO41" s="26"/>
+      <c r="AP41" s="26"/>
+      <c r="AQ41" s="26"/>
+      <c r="AR41" s="25">
         <v>0</v>
       </c>
-      <c r="AS40" s="25">
+      <c r="AS41" s="25">
         <v>0</v>
       </c>
-      <c r="AT40" s="25">
+      <c r="AT41" s="25">
         <v>0</v>
       </c>
-      <c r="AU40" s="25">
+      <c r="AU41" s="25">
         <v>0</v>
       </c>
-      <c r="AV40" s="52">
+      <c r="AV41" s="52">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AW40" s="52">
+      <c r="AW41" s="52">
         <v>0</v>
       </c>
-      <c r="AX40" s="52">
+      <c r="AX41" s="52">
         <v>0</v>
       </c>
-      <c r="AY40" s="25"/>
-      <c r="AZ40" s="23"/>
-      <c r="BA40" s="25"/>
-      <c r="BB40" s="25"/>
-      <c r="BC40" s="27"/>
-      <c r="BD40" s="25"/>
-      <c r="BE40" s="28"/>
-      <c r="BF40" s="25"/>
-      <c r="BG40" s="57" t="str">
+      <c r="AY41" s="25"/>
+      <c r="AZ41" s="23"/>
+      <c r="BA41" s="25"/>
+      <c r="BB41" s="25"/>
+      <c r="BC41" s="27"/>
+      <c r="BD41" s="25"/>
+      <c r="BE41" s="28"/>
+      <c r="BF41" s="25"/>
+      <c r="BG41" s="57" t="str">
         <f t="shared" si="2"/>
         <v>description: "IRF", note: "Внутренняя неисправность", group: "measurement", minValue: null, maxValue: null, step: null, units: "null", defaultValue: null, eventRegistration: 0</v>
       </c>
-      <c r="BH40" s="30"/>
-    </row>
-    <row r="41" spans="1:60" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" s="1"/>
-      <c r="B41" s="1"/>
-      <c r="C41" s="1"/>
-      <c r="D41" s="1"/>
-      <c r="R41" s="3"/>
-      <c r="S41" s="4"/>
-      <c r="T41" s="4"/>
-      <c r="U41" s="4"/>
-      <c r="V41" s="4"/>
-      <c r="W41" s="4"/>
-      <c r="X41" s="4"/>
-      <c r="Y41" s="4"/>
-      <c r="Z41" s="1"/>
-      <c r="AA41" s="4"/>
-      <c r="AB41" s="4"/>
-      <c r="AC41" s="4"/>
-      <c r="AD41" s="4"/>
-      <c r="AE41" s="4"/>
-      <c r="AF41" s="4"/>
-      <c r="AG41" s="4"/>
-      <c r="AH41" s="1"/>
-      <c r="AI41" s="4"/>
-      <c r="AR41" s="4"/>
-      <c r="AS41" s="4"/>
-      <c r="AT41" s="4"/>
-      <c r="AU41" s="4"/>
-      <c r="AV41" s="4"/>
-      <c r="AW41" s="4"/>
-      <c r="AX41" s="4"/>
-      <c r="AY41" s="4"/>
-      <c r="AZ41" s="4"/>
-      <c r="BA41" s="4"/>
-      <c r="BB41" s="33"/>
-      <c r="BC41" s="4"/>
-      <c r="BD41" s="33"/>
-      <c r="BE41" s="4"/>
-      <c r="BF41" s="4"/>
-      <c r="BG41" s="1"/>
-      <c r="BH41" s="1"/>
+      <c r="BH41" s="30"/>
     </row>
     <row r="42" spans="1:60" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
@@ -24752,13 +24928,13 @@
       <c r="AG93" s="4"/>
       <c r="AH93" s="1"/>
       <c r="AI93" s="4"/>
-      <c r="AR93" s="1"/>
-      <c r="AS93" s="1"/>
-      <c r="AT93" s="1"/>
-      <c r="AU93" s="1"/>
-      <c r="AV93" s="1"/>
-      <c r="AW93" s="1"/>
-      <c r="AX93" s="1"/>
+      <c r="AR93" s="4"/>
+      <c r="AS93" s="4"/>
+      <c r="AT93" s="4"/>
+      <c r="AU93" s="4"/>
+      <c r="AV93" s="4"/>
+      <c r="AW93" s="4"/>
+      <c r="AX93" s="4"/>
       <c r="AY93" s="4"/>
       <c r="AZ93" s="4"/>
       <c r="BA93" s="4"/>
@@ -24792,7 +24968,7 @@
       <c r="AF94" s="4"/>
       <c r="AG94" s="4"/>
       <c r="AH94" s="1"/>
-      <c r="AI94" s="1"/>
+      <c r="AI94" s="4"/>
       <c r="AR94" s="1"/>
       <c r="AS94" s="1"/>
       <c r="AT94" s="1"/>
@@ -25235,13 +25411,13 @@
       <c r="X105" s="4"/>
       <c r="Y105" s="4"/>
       <c r="Z105" s="1"/>
-      <c r="AA105" s="1"/>
-      <c r="AB105" s="1"/>
-      <c r="AC105" s="1"/>
-      <c r="AD105" s="1"/>
-      <c r="AE105" s="1"/>
-      <c r="AF105" s="1"/>
-      <c r="AG105" s="1"/>
+      <c r="AA105" s="4"/>
+      <c r="AB105" s="4"/>
+      <c r="AC105" s="4"/>
+      <c r="AD105" s="4"/>
+      <c r="AE105" s="4"/>
+      <c r="AF105" s="4"/>
+      <c r="AG105" s="4"/>
       <c r="AH105" s="1"/>
       <c r="AI105" s="1"/>
       <c r="AR105" s="1"/>
@@ -26328,6 +26504,47 @@
       <c r="BG131" s="1"/>
       <c r="BH131" s="1"/>
     </row>
+    <row r="132" spans="1:60" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A132" s="1"/>
+      <c r="B132" s="1"/>
+      <c r="C132" s="1"/>
+      <c r="D132" s="1"/>
+      <c r="R132" s="3"/>
+      <c r="S132" s="4"/>
+      <c r="T132" s="4"/>
+      <c r="U132" s="4"/>
+      <c r="V132" s="4"/>
+      <c r="W132" s="4"/>
+      <c r="X132" s="4"/>
+      <c r="Y132" s="4"/>
+      <c r="Z132" s="1"/>
+      <c r="AA132" s="1"/>
+      <c r="AB132" s="1"/>
+      <c r="AC132" s="1"/>
+      <c r="AD132" s="1"/>
+      <c r="AE132" s="1"/>
+      <c r="AF132" s="1"/>
+      <c r="AG132" s="1"/>
+      <c r="AH132" s="1"/>
+      <c r="AI132" s="1"/>
+      <c r="AR132" s="1"/>
+      <c r="AS132" s="1"/>
+      <c r="AT132" s="1"/>
+      <c r="AU132" s="1"/>
+      <c r="AV132" s="1"/>
+      <c r="AW132" s="1"/>
+      <c r="AX132" s="1"/>
+      <c r="AY132" s="4"/>
+      <c r="AZ132" s="4"/>
+      <c r="BA132" s="4"/>
+      <c r="BB132" s="33"/>
+      <c r="BC132" s="4"/>
+      <c r="BD132" s="33"/>
+      <c r="BE132" s="4"/>
+      <c r="BF132" s="4"/>
+      <c r="BG132" s="1"/>
+      <c r="BH132" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="AZ1:BF1"/>
@@ -26433,15 +26650,15 @@
       <c r="AW1" s="6"/>
       <c r="AX1" s="6"/>
       <c r="AY1" s="8"/>
-      <c r="AZ1" s="59" t="s">
+      <c r="AZ1" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="BA1" s="60"/>
-      <c r="BB1" s="60"/>
-      <c r="BC1" s="60"/>
-      <c r="BD1" s="60"/>
-      <c r="BE1" s="60"/>
-      <c r="BF1" s="60"/>
+      <c r="BA1" s="67"/>
+      <c r="BB1" s="67"/>
+      <c r="BC1" s="67"/>
+      <c r="BD1" s="67"/>
+      <c r="BE1" s="67"/>
+      <c r="BF1" s="67"/>
     </row>
     <row r="2" spans="1:16379" s="17" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
@@ -26585,14 +26802,14 @@
       <c r="AU2" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="AV2" s="65" t="s">
-        <v>223</v>
-      </c>
-      <c r="AW2" s="65" t="s">
-        <v>224</v>
-      </c>
-      <c r="AX2" s="65" t="s">
-        <v>225</v>
+      <c r="AV2" s="63" t="s">
+        <v>220</v>
+      </c>
+      <c r="AW2" s="63" t="s">
+        <v>221</v>
+      </c>
+      <c r="AX2" s="63" t="s">
+        <v>222</v>
       </c>
       <c r="AY2" s="14"/>
       <c r="AZ2" s="13" t="s">
@@ -42942,21 +43159,21 @@
     </row>
     <row r="3" spans="1:16379" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="18"/>
-      <c r="B3" s="64" t="s">
-        <v>222</v>
+      <c r="B3" s="62" t="s">
+        <v>219</v>
       </c>
       <c r="C3" s="25"/>
       <c r="D3" s="32" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="F3" s="34" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="G3" s="34" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="H3" s="8"/>
       <c r="I3" s="21">
@@ -42968,7 +43185,7 @@
         <v>Пуск (имп)</v>
       </c>
       <c r="K3" s="24" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="L3" s="22" t="s">
         <v>62</v>
@@ -43040,13 +43257,13 @@
       <c r="AU3" s="25">
         <v>1</v>
       </c>
-      <c r="AV3" s="66">
+      <c r="AV3" s="64">
         <v>1</v>
       </c>
-      <c r="AW3" s="66">
+      <c r="AW3" s="64">
         <v>1</v>
       </c>
-      <c r="AX3" s="66">
+      <c r="AX3" s="64">
         <v>1</v>
       </c>
       <c r="AY3" s="23"/>
@@ -43064,21 +43281,21 @@
     </row>
     <row r="4" spans="1:16379" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="18"/>
-      <c r="B4" s="64" t="s">
-        <v>222</v>
+      <c r="B4" s="62" t="s">
+        <v>219</v>
       </c>
       <c r="C4" s="25"/>
       <c r="D4" s="32" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F4" s="34" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="G4" s="34" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="H4" s="8"/>
       <c r="I4" s="21">
@@ -43090,7 +43307,7 @@
         <v>Пуск</v>
       </c>
       <c r="K4" s="24" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="L4" s="22" t="s">
         <v>62</v>
@@ -43162,13 +43379,13 @@
       <c r="AU4" s="25">
         <v>1</v>
       </c>
-      <c r="AV4" s="66">
+      <c r="AV4" s="64">
         <v>1</v>
       </c>
-      <c r="AW4" s="66">
+      <c r="AW4" s="64">
         <v>1</v>
       </c>
-      <c r="AX4" s="66">
+      <c r="AX4" s="64">
         <v>1</v>
       </c>
       <c r="AY4" s="23"/>
@@ -43290,15 +43507,15 @@
       <c r="AW1" s="6"/>
       <c r="AX1" s="6"/>
       <c r="AY1" s="8"/>
-      <c r="AZ1" s="59" t="s">
+      <c r="AZ1" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="BA1" s="60"/>
-      <c r="BB1" s="60"/>
-      <c r="BC1" s="60"/>
-      <c r="BD1" s="60"/>
-      <c r="BE1" s="60"/>
-      <c r="BF1" s="60"/>
+      <c r="BA1" s="67"/>
+      <c r="BB1" s="67"/>
+      <c r="BC1" s="67"/>
+      <c r="BD1" s="67"/>
+      <c r="BE1" s="67"/>
+      <c r="BF1" s="67"/>
     </row>
     <row r="2" spans="1:16379" s="17" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
@@ -59800,23 +60017,23 @@
     <row r="3" spans="1:16379" s="31" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="18"/>
       <c r="B3" s="18" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C3" s="19"/>
       <c r="D3" s="32" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E3" s="21" t="s">
+        <v>156</v>
+      </c>
+      <c r="F3" s="21" t="s">
+        <v>157</v>
+      </c>
+      <c r="G3" s="21" t="s">
+        <v>158</v>
+      </c>
+      <c r="H3" s="21" t="s">
         <v>159</v>
-      </c>
-      <c r="F3" s="21" t="s">
-        <v>160</v>
-      </c>
-      <c r="G3" s="21" t="s">
-        <v>161</v>
-      </c>
-      <c r="H3" s="21" t="s">
-        <v>162</v>
       </c>
       <c r="I3" s="21">
         <f t="shared" ref="I3:I9" si="0">LEN(F3)</f>
@@ -59827,7 +60044,7 @@
         <v>Контр_цепей</v>
       </c>
       <c r="K3" s="18" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="L3" s="22" t="s">
         <v>62</v>
@@ -59906,7 +60123,7 @@
         <v>0</v>
       </c>
       <c r="AW3" s="25" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="AX3" s="25"/>
       <c r="AY3" s="23"/>
@@ -59925,23 +60142,23 @@
     <row r="4" spans="1:16379" s="31" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="18"/>
       <c r="B4" s="18" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C4" s="19"/>
       <c r="D4" s="32" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="F4" s="21" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="H4" s="21" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I4" s="21">
         <f t="shared" si="0"/>
@@ -59952,7 +60169,7 @@
         <v>Контр_вывода_БИ</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="L4" s="22" t="s">
         <v>62</v>
@@ -60031,7 +60248,7 @@
         <v>0</v>
       </c>
       <c r="AW4" s="25" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="AX4" s="25"/>
       <c r="AY4" s="23"/>
@@ -60050,23 +60267,23 @@
     <row r="5" spans="1:16379" s="31" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="18"/>
       <c r="B5" s="18" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C5" s="19"/>
       <c r="D5" s="32" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="F5" s="21" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="G5" s="21" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="H5" s="21" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I5" s="21">
         <f t="shared" si="0"/>
@@ -60077,7 +60294,7 @@
         <v>Контр_ОТ_сигн</v>
       </c>
       <c r="K5" s="18" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="L5" s="22" t="s">
         <v>62</v>
@@ -60156,7 +60373,7 @@
         <v>0</v>
       </c>
       <c r="AW5" s="25" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="AX5" s="25"/>
       <c r="AY5" s="23"/>
@@ -60175,23 +60392,23 @@
     <row r="6" spans="1:16379" s="31" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="18"/>
       <c r="B6" s="18" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C6" s="19"/>
       <c r="D6" s="32" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F6" s="21" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="H6" s="21" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I6" s="21">
         <f t="shared" si="0"/>
@@ -60202,7 +60419,7 @@
         <v>Контр_Неиспр_КА</v>
       </c>
       <c r="K6" s="18" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="L6" s="22" t="s">
         <v>62</v>
@@ -60281,7 +60498,7 @@
         <v>0</v>
       </c>
       <c r="AW6" s="25" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="AX6" s="25"/>
       <c r="AY6" s="23"/>
@@ -60300,23 +60517,23 @@
     <row r="7" spans="1:16379" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="18"/>
       <c r="B7" s="18" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C7" s="19"/>
       <c r="D7" s="32" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="H7" s="21" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I7" s="21">
         <f t="shared" si="0"/>
@@ -60327,7 +60544,7 @@
         <v>Контр_прев_вр_пер</v>
       </c>
       <c r="K7" s="18" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="L7" s="22" t="s">
         <v>62</v>
@@ -60406,7 +60623,7 @@
         <v>0</v>
       </c>
       <c r="AW7" s="25" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="AX7" s="25"/>
       <c r="AY7" s="23"/>
@@ -60425,23 +60642,23 @@
     <row r="8" spans="1:16379" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="18"/>
       <c r="B8" s="18" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C8" s="19"/>
       <c r="D8" s="32" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="F8" s="21" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="H8" s="21" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I8" s="21">
         <f t="shared" si="0"/>
@@ -60452,7 +60669,7 @@
         <v>Контр_общ_вн_сигн</v>
       </c>
       <c r="K8" s="18" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="L8" s="22" t="s">
         <v>62</v>
@@ -60531,7 +60748,7 @@
         <v>0</v>
       </c>
       <c r="AW8" s="25" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="AX8" s="25"/>
       <c r="AY8" s="23"/>
@@ -60550,23 +60767,23 @@
     <row r="9" spans="1:16379" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="18"/>
       <c r="B9" s="18" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C9" s="19"/>
       <c r="D9" s="32" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F9" s="21" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="H9" s="21" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I9" s="21">
         <f t="shared" si="0"/>
@@ -60577,7 +60794,7 @@
         <v>Контр_пол_ав_дебл</v>
       </c>
       <c r="K9" s="18" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="L9" s="22" t="s">
         <v>62</v>
@@ -60656,7 +60873,7 @@
         <v>0</v>
       </c>
       <c r="AW9" s="25" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="AX9" s="25"/>
       <c r="AY9" s="23"/>
@@ -60693,23 +60910,23 @@
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="39" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B3" s="40" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B4" s="41">
         <v>580</v>
@@ -60717,7 +60934,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B5" s="42" t="s">
         <v>64</v>
@@ -60725,47 +60942,47 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="43" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="43" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B7" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" s="62" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="61" t="s">
-        <v>219</v>
+    <row r="8" spans="1:2" s="60" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="59" t="s">
+        <v>216</v>
       </c>
       <c r="B8" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
     </row>
-    <row r="9" spans="1:2" s="62" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="61" t="s">
-        <v>221</v>
-      </c>
-      <c r="B9" s="61"/>
+    <row r="9" spans="1:2" s="60" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="59" t="s">
+        <v>218</v>
+      </c>
+      <c r="B9" s="59"/>
     </row>
-    <row r="10" spans="1:2" s="62" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="63" t="s">
-        <v>151</v>
+    <row r="10" spans="1:2" s="60" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="61" t="s">
+        <v>148</v>
       </c>
       <c r="B10" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
     </row>
-    <row r="11" spans="1:2" s="62" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="61" t="s">
-        <v>221</v>
-      </c>
-      <c r="B11" s="61"/>
+    <row r="11" spans="1:2" s="60" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="59" t="s">
+        <v>218</v>
+      </c>
+      <c r="B11" s="59"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>